<commit_message>
Streamline the campaign home and harden credibility.
Collapse duplicate CTAs and vendor chapters onto dedicated pages, remove parked For-Flock HTML and overclaim edges, and keep deep links scrolling to the right council and archive sections.
</commit_message>
<xml_diff>
--- a/docs/Flock_Safety_ALPR_Misuse_Master_Database.xlsx
+++ b/docs/Flock_Safety_ALPR_Misuse_Master_Database.xlsx
@@ -595,7 +595,6 @@
       <c r="P2" t="n">
         <v>2026</v>
       </c>
-      <c r="R2" t="inlineStr"/>
       <c r="S2" t="inlineStr">
         <is>
           <t>Terminated / Resigned (Employment Fallout)</t>
@@ -679,7 +678,6 @@
       <c r="P3" t="n">
         <v>2026</v>
       </c>
-      <c r="R3" t="inlineStr"/>
       <c r="S3" t="inlineStr">
         <is>
           <t>Terminated / Resigned &amp; Criminally Charged</t>
@@ -856,7 +854,6 @@
       <c r="P5" t="n">
         <v>2026</v>
       </c>
-      <c r="R5" t="inlineStr"/>
       <c r="S5" t="inlineStr">
         <is>
           <t>Terminated / Resigned &amp; Criminally Charged</t>
@@ -940,7 +937,6 @@
       <c r="P6" t="n">
         <v>2026</v>
       </c>
-      <c r="R6" t="inlineStr"/>
       <c r="S6" t="inlineStr">
         <is>
           <t>Terminated / Resigned &amp; Criminally Charged</t>
@@ -1024,7 +1020,6 @@
       <c r="P7" t="n">
         <v>2026</v>
       </c>
-      <c r="R7" t="inlineStr"/>
       <c r="S7" t="inlineStr">
         <is>
           <t>Terminated / Resigned &amp; Criminally Charged</t>
@@ -1108,7 +1103,6 @@
       <c r="P8" t="n">
         <v>2026</v>
       </c>
-      <c r="R8" t="inlineStr"/>
       <c r="S8" t="inlineStr">
         <is>
           <t>Criminally Charged / Indicted</t>
@@ -1192,7 +1186,6 @@
       <c r="P9" t="n">
         <v>2026</v>
       </c>
-      <c r="R9" t="inlineStr"/>
       <c r="S9" t="inlineStr">
         <is>
           <t>Criminally Charged / Indicted</t>
@@ -1276,7 +1269,6 @@
       <c r="P10" t="n">
         <v>2026</v>
       </c>
-      <c r="R10" t="inlineStr"/>
       <c r="S10" t="inlineStr">
         <is>
           <t>Internal Disciplinary Action / Other</t>
@@ -1360,7 +1352,6 @@
       <c r="P11" t="n">
         <v>2026</v>
       </c>
-      <c r="R11" t="inlineStr"/>
       <c r="S11" t="inlineStr">
         <is>
           <t>Terminated / Resigned (Employment Fallout)</t>
@@ -1444,7 +1435,6 @@
       <c r="P12" t="n">
         <v>2026</v>
       </c>
-      <c r="R12" t="inlineStr"/>
       <c r="S12" t="inlineStr">
         <is>
           <t>Criminally Charged / Indicted</t>
@@ -1528,7 +1518,6 @@
       <c r="P13" t="n">
         <v>2026</v>
       </c>
-      <c r="R13" t="inlineStr"/>
       <c r="S13" t="inlineStr">
         <is>
           <t>Criminally Charged / Indicted</t>
@@ -1612,7 +1601,6 @@
       <c r="P14" t="n">
         <v>2026</v>
       </c>
-      <c r="R14" t="inlineStr"/>
       <c r="S14" t="inlineStr">
         <is>
           <t>Civil Lawsuit / Settlement / Dismissed Stop</t>
@@ -1696,7 +1684,6 @@
       <c r="P15" t="n">
         <v>2026</v>
       </c>
-      <c r="R15" t="inlineStr"/>
       <c r="S15" t="inlineStr">
         <is>
           <t>Criminally Charged / Indicted</t>
@@ -1871,7 +1858,6 @@
       <c r="P17" t="n">
         <v>2026</v>
       </c>
-      <c r="R17" t="inlineStr"/>
       <c r="S17" t="inlineStr">
         <is>
           <t>Civil Lawsuit / Settlement / Dismissed Stop</t>
@@ -1955,7 +1941,6 @@
       <c r="P18" t="n">
         <v>2026</v>
       </c>
-      <c r="R18" t="inlineStr"/>
       <c r="S18" t="inlineStr">
         <is>
           <t>Civil Lawsuit / Settlement / Dismissed Stop</t>
@@ -2039,7 +2024,6 @@
       <c r="P19" t="n">
         <v>2025</v>
       </c>
-      <c r="R19" t="inlineStr"/>
       <c r="S19" t="inlineStr">
         <is>
           <t>Terminated / Resigned &amp; Criminally Charged</t>
@@ -2123,7 +2107,6 @@
       <c r="P20" t="n">
         <v>2025</v>
       </c>
-      <c r="R20" t="inlineStr"/>
       <c r="S20" t="inlineStr">
         <is>
           <t>Terminated / Resigned &amp; Criminally Charged</t>
@@ -2207,7 +2190,6 @@
       <c r="P21" t="n">
         <v>2025</v>
       </c>
-      <c r="R21" t="inlineStr"/>
       <c r="S21" t="inlineStr">
         <is>
           <t>Terminated / Resigned &amp; Criminally Charged</t>
@@ -2291,7 +2273,6 @@
       <c r="P22" t="n">
         <v>2025</v>
       </c>
-      <c r="R22" t="inlineStr"/>
       <c r="S22" t="inlineStr">
         <is>
           <t>Criminally Charged / Indicted</t>
@@ -2375,7 +2356,6 @@
       <c r="P23" t="n">
         <v>2025</v>
       </c>
-      <c r="R23" t="inlineStr"/>
       <c r="S23" t="inlineStr">
         <is>
           <t>Summons Voided / Officer Discipline</t>
@@ -2459,7 +2439,6 @@
       <c r="P24" t="n">
         <v>2025</v>
       </c>
-      <c r="R24" t="inlineStr"/>
       <c r="S24" t="inlineStr">
         <is>
           <t>Resigned &amp; Criminally Charged</t>
@@ -2543,7 +2522,6 @@
       <c r="P25" t="n">
         <v>2025</v>
       </c>
-      <c r="R25" t="inlineStr"/>
       <c r="S25" t="inlineStr">
         <is>
           <t>Internal Disciplinary Action / Other</t>
@@ -2627,7 +2605,6 @@
       <c r="P26" t="n">
         <v>2025</v>
       </c>
-      <c r="R26" t="inlineStr"/>
       <c r="S26" t="inlineStr">
         <is>
           <t>Civil Lawsuit / Settlement / Dismissed Stop</t>
@@ -2711,7 +2688,6 @@
       <c r="P27" t="n">
         <v>2025</v>
       </c>
-      <c r="R27" t="inlineStr"/>
       <c r="S27" t="inlineStr">
         <is>
           <t>Internal Disciplinary Action / Other</t>
@@ -2886,7 +2862,6 @@
       <c r="P29" t="n">
         <v>2024</v>
       </c>
-      <c r="R29" t="inlineStr"/>
       <c r="S29" t="inlineStr">
         <is>
           <t>Terminated / Resigned (Employment Fallout)</t>
@@ -3078,7 +3053,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>FLK-2024-030</t>
+          <t>ALPR-2024-030</t>
         </is>
       </c>
       <c r="B32" t="n">
@@ -3152,7 +3127,6 @@
       <c r="P32" t="n">
         <v>2024</v>
       </c>
-      <c r="R32" t="inlineStr"/>
       <c r="S32" t="inlineStr">
         <is>
           <t>Relieved of Duty / Under Investigation</t>
@@ -3236,7 +3210,6 @@
       <c r="P33" t="n">
         <v>2024</v>
       </c>
-      <c r="R33" t="inlineStr"/>
       <c r="S33" t="inlineStr">
         <is>
           <t>Internal Disciplinary Action / Other</t>
@@ -3502,7 +3475,6 @@
       <c r="P36" t="n">
         <v>2023</v>
       </c>
-      <c r="R36" t="inlineStr"/>
       <c r="S36" t="inlineStr">
         <is>
           <t>Terminated / Resigned (Employment Fallout)</t>
@@ -3677,7 +3649,6 @@
       <c r="P38" t="n">
         <v>2021</v>
       </c>
-      <c r="R38" t="inlineStr"/>
       <c r="S38" t="inlineStr">
         <is>
           <t>Criminally Charged / Indicted</t>
@@ -3761,7 +3732,6 @@
       <c r="P39" t="n">
         <v>2020</v>
       </c>
-      <c r="R39" t="inlineStr"/>
       <c r="S39" t="inlineStr">
         <is>
           <t>Internal Disciplinary Action / Other</t>
@@ -3845,7 +3815,6 @@
       <c r="P40" t="n">
         <v>2020</v>
       </c>
-      <c r="R40" t="inlineStr"/>
       <c r="S40" t="inlineStr">
         <is>
           <t>Civil Lawsuit / Settlement / Dismissed Stop</t>

</xml_diff>

<commit_message>
Add Bibb County Flock audit investigation to the misuse dossier.
Document the sheriff’s Internal Affairs review of three flagged queries, bump verified misuse tallies to 53, and regenerate PDF/Excel exports.
</commit_message>
<xml_diff>
--- a/docs/Flock_Safety_ALPR_Misuse_Master_Database.xlsx
+++ b/docs/Flock_Safety_ALPR_Misuse_Master_Database.xlsx
@@ -450,7 +450,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S53"/>
+  <dimension ref="A1:S54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -5339,6 +5339,99 @@
         </is>
       </c>
     </row>
+    <row r="54">
+      <c r="A54" s="2" t="inlineStr">
+        <is>
+          <t>FLK-2026-031</t>
+        </is>
+      </c>
+      <c r="B54" s="2" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="C54" s="2" t="inlineStr">
+        <is>
+          <t>GA</t>
+        </is>
+      </c>
+      <c r="D54" s="2" t="inlineStr">
+        <is>
+          <t>Bibb County Sheriff’s Office</t>
+        </is>
+      </c>
+      <c r="E54" s="2" t="inlineStr">
+        <is>
+          <t>Deputies under review (unnamed; three flagged queries)</t>
+        </is>
+      </c>
+      <c r="F54" s="2" t="inlineStr">
+        <is>
+          <t>Flock Safety</t>
+        </is>
+      </c>
+      <c r="G54" s="2" t="inlineStr">
+        <is>
+          <t>Unauthorized Access / Personal Tracking</t>
+        </is>
+      </c>
+      <c r="H54" s="2" t="inlineStr">
+        <is>
+          <t>Three separate queries flagged by monthly audit algorithm</t>
+        </is>
+      </c>
+      <c r="I54" s="2" t="inlineStr">
+        <is>
+          <t>On August 3–4, 2026, the Bibb County Sheriff’s Office said its routine monthly Flock audit returned three separate queries flagged as problematic by Flock’s auditing algorithm. Internal Affairs is reviewing whether any deputies violated policy. Officials said no deputies had been terminated or placed on administrative leave, but those under review had Flock access suspended pending the outcome. The agency said it would publicly disclose confirmed findings of misuse when investigations finish. Allegations under investigation, not findings of guilt.</t>
+        </is>
+      </c>
+      <c r="J54" s="2" t="inlineStr">
+        <is>
+          <t>Monthly agency Flock audit / Audit Assistance algorithm</t>
+        </is>
+      </c>
+      <c r="K54" s="2" t="inlineStr">
+        <is>
+          <t>Internal Affairs investigations open; Flock access suspended for deputies under review; no firings or leave announced as of Aug. 3–4 reporting.</t>
+        </is>
+      </c>
+      <c r="L54" s="2" t="inlineStr">
+        <is>
+          <t>Georgia Public Broadcasting; WGXA; Macon Telegraph; 41NBC</t>
+        </is>
+      </c>
+      <c r="M54" s="2" t="inlineStr">
+        <is>
+          <t>https://www.gpb.org/news/2026/08/04/bibb-county-sheriffs-office-launches-investigation-for-potential-misuse-of-flock</t>
+        </is>
+      </c>
+      <c r="N54" s="2" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="O54" s="2" t="inlineStr">
+        <is>
+          <t>Agency statement carried by GPB / WGXA / Macon Telegraph / 41NBC; names and query details withheld; investigations active.</t>
+        </is>
+      </c>
+      <c r="P54" s="2" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="Q54" s="2" t="inlineStr"/>
+      <c r="R54" s="2" t="inlineStr">
+        <is>
+          <t>Investigations announced Aug. 3–4, 2026; outcomes pending.</t>
+        </is>
+      </c>
+      <c r="S54" s="2" t="inlineStr">
+        <is>
+          <t>Under Investigation / Pending</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>